<commit_message>
docs: align API contracts and restructure testing examples
</commit_message>
<xml_diff>
--- a/pruebas/3.2-Casos-de-Prueba-BrainSort.xlsx
+++ b/pruebas/3.2-Casos-de-Prueba-BrainSort.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Prueba'!$A$1:$K$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Prueba'!$A$1:$K$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Equivalencia y Limites'!$A$1:$L$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trazabilidad'!$A$1:$D$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automatizacion'!$A$1:$E$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trazabilidad'!$A$1:$D$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automatizacion'!$A$1:$E$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Resumen'!$A$1:$B$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1227,7 +1227,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Unitaria</t>
+          <t>Unitaria/E2E</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Retorna descripcion completa, complejidad, categoria, tags y pseudocode</t>
+          <t>Retorna descripcion completa, complejidad, categoria, tags y pseudocode normalizado line/text/indent</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>src/algorithms/algorithms.service.spec.ts</t>
+          <t>src/algorithms/algorithms.service.spec.ts; test/algorithms.e2e-spec.ts</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>correcto=true, puntosGanados, feedbackPositivo</t>
+          <t>correcto=true, puntosGanados, feedback y feedbackPositivo</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>correcto=false, puntosGanados=0, feedbackNegativo</t>
+          <t>correcto=false, puntosGanados=0, feedback y feedbackNegativo</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Unitaria</t>
+          <t>Unitaria/E2E</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Retorna meta,pseudocode,ejercicios</t>
+          <t>Retorna algoritmoId, version, meta, pseudocode y ejercicios</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>src/offline/offline.service.spec.ts</t>
+          <t>src/offline/offline.service.spec.ts; test/learning-support.e2e-spec.ts</t>
         </is>
       </c>
     </row>
@@ -2924,8 +2924,293 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>CP-LRN-001</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Soporte Aprendizaje</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>RF-DIAG/RF-RUTA</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Evaluar diagnostico y consultar ruta HTTP</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Token valido y preguntas diagnosticas</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>GET preguntas, POST evaluar, GET ruta</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Respuestas 200/201 y ruta con algoritmos sugeridos</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>test/learning-support.e2e-spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>CP-LRN-002</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Insignias</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>RF-INS</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Consultar insignias HTTP</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Token valido</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/insignias y /api/insignias/me</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Lista insignias disponibles y estado del usuario</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>test/learning-support.e2e-spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>CP-LRN-003</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>RF-OFF</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Listar y descargar modulo offline HTTP</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Token valido y algoritmos activos</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/modules/offline y /download</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Retorna meta, pseudocode y ejercicios del modulo</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>test/learning-support.e2e-spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>CP-LRN-004</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Seguridad API</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>RF-AUTH</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Proteger endpoints de aprendizaje</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Sin token JWT</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>GET endpoints protegidos</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Retorna 401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Critica</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>test/learning-support.e2e-spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-SVC-001</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Contratos FE</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>RF-CONTRATOS</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Consumir contratos API desde frontend</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>apiClient mockeado</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>ranking, sync, offline, ejercicios</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Valida endpoints y forma ranking/total, completada, algoritmoId/version y feedback</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>src/services/__tests__/contract-shapes.test.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K43"/>
+  <autoFilter ref="A1:K48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3417,7 +3702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3693,17 +3978,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>RF-DIAG</t>
+          <t>RF-AUTH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Diagnostico</t>
+          <t>Seguridad API</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>CP-DIAG-001, CP-DIAG-002</t>
+          <t>CP-LRN-004</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -3715,17 +4000,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>RF-EJR</t>
+          <t>RF-CONTRATOS</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ejercicios</t>
+          <t>Contratos FE</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>CP-EJR-001, CP-EJR-002, CP-EJR-003, CP-EJR-004, CP-EJR-005</t>
+          <t>CP-FE-SVC-001</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -3737,17 +4022,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>RF-INS</t>
+          <t>RF-DIAG</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Insignias</t>
+          <t>Diagnostico</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>CP-INS-001, CP-INS-002</t>
+          <t>CP-DIAG-001, CP-DIAG-002</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -3759,17 +4044,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>RF-OFF</t>
+          <t>RF-DIAG/RF-RUTA</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Soporte Aprendizaje</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>CP-OFF-001, CP-OFF-002</t>
+          <t>CP-LRN-001</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -3781,17 +4066,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>RF-PRG</t>
+          <t>RF-EJR</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Progreso</t>
+          <t>Ejercicios</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>CP-PRG-001, CP-PRG-002, CP-PRG-003</t>
+          <t>CP-EJR-001, CP-EJR-002, CP-EJR-003, CP-EJR-004, CP-EJR-005</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -3803,17 +4088,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>RF-RUTA</t>
+          <t>RF-INS</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Ruta Aprendizaje</t>
+          <t>Insignias</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>CP-RUTA-001</t>
+          <t>CP-INS-001, CP-INS-002, CP-LRN-002</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -3825,17 +4110,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>RF-SYNC</t>
+          <t>RF-OFF</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Sync</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>CP-SYNC-001</t>
+          <t>CP-OFF-001, CP-OFF-002, CP-LRN-003</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -3847,27 +4132,93 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>RF-PRG</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Progreso</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>CP-PRG-001, CP-PRG-002, CP-PRG-003</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Automatizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>RF-RUTA</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Ruta Aprendizaje</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>CP-RUTA-001</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Automatizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>RF-SYNC</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Sync</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>CP-SYNC-001</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Automatizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>RF-USR</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Usuarios</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>CP-USR-001, CP-USR-002</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Automatizado</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D20"/>
+  <autoFilter ref="A1:D23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3878,7 +4229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3932,11 +4283,11 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Registro, login usuario/admin, refresh, errores</t>
+          <t>Registro, login usuario/admin, refresh usuario/admin, errores</t>
         </is>
       </c>
     </row>
@@ -4232,11 +4583,11 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Biblioteca y detalle</t>
+          <t>Biblioteca, detalle y pseudocode normalizado</t>
         </is>
       </c>
     </row>
@@ -4323,7 +4674,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>test/app.e2e-spec.ts</t>
+          <t>test/learning-support.e2e-spec.ts</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -4332,36 +4683,36 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Health/ruta raiz</t>
+          <t>Diagnostico, ruta, insignias y offline</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>packages/core/src/engines/__tests__/bubble-sort.test.ts</t>
+          <t>test/app.e2e-spec.ts</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Unitaria</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Bubble Sort</t>
+          <t>Health/ruta raiz</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4724,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>packages/core/src/engines/__tests__/selection-sort.test.ts</t>
+          <t>packages/core/src/engines/__tests__/bubble-sort.test.ts</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -4386,7 +4737,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Selection Sort</t>
+          <t>Bubble Sort</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4749,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>packages/core/src/engines/__tests__/insertion-sort.test.ts</t>
+          <t>packages/core/src/engines/__tests__/selection-sort.test.ts</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -4411,7 +4762,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Insertion Sort</t>
+          <t>Selection Sort</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4774,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>packages/core/src/engines/__tests__/merge-sort.test.ts</t>
+          <t>packages/core/src/engines/__tests__/insertion-sort.test.ts</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -4436,7 +4787,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Merge Sort</t>
+          <t>Insertion Sort</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4799,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>packages/core/src/math/__tests__/math.test.ts</t>
+          <t>packages/core/src/engines/__tests__/merge-sort.test.ts</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -4457,11 +4808,11 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Escalas, coordenadas, transiciones</t>
+          <t>Merge Sort</t>
         </is>
       </c>
     </row>
@@ -4473,25 +4824,75 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
+          <t>packages/core/src/math/__tests__/math.test.ts</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Escalas, coordenadas, transiciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
           <t>packages/core/src/validators/__tests__/dataset.test.ts</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Unitaria</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="n">
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Validacion de datasets</t>
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>src/services/__tests__/contract-shapes.test.ts</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Contratos frontend para ranking, ejercicios, offline y sync</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E24"/>
+  <autoFilter ref="A1:E26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4528,7 +4929,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -4538,7 +4939,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>152</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4">
@@ -4549,7 +4950,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>11 suites / 93 tests pasados</t>
+          <t>11 suites / 94 tests pasados</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4962,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>6 suites / 28 tests pasados</t>
+          <t>7 suites / 33 tests pasados</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4974,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>6 suites / 31 tests pasados</t>
+          <t>7 suites / 35 tests pasados</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4986,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>feature/unit-tests-qa</t>
+          <t>API feature/unit-tests-qa; APP feature/contract-consistency-fixes</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4998,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>fecbfca test: strengthen service coverage review</t>
+          <t>86b4413 base + cambios locales de contratos</t>
         </is>
       </c>
     </row>
@@ -4609,7 +5010,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>077d316 fix: align simulation canvas color token</t>
+          <t>b66290b base dev + cambios locales de contratos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: actualizar documentos de pruebas y especificaciones UI/UX
</commit_message>
<xml_diff>
--- a/pruebas/3.2-Casos-de-Prueba-BrainSort.xlsx
+++ b/pruebas/3.2-Casos-de-Prueba-BrainSort.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Prueba'!$A$1:$K$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Prueba'!$A$1:$K$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Equivalencia y Limites'!$A$1:$L$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trazabilidad'!$A$1:$D$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automatizacion'!$A$1:$E$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trazabilidad'!$A$1:$D$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automatizacion'!$A$1:$E$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Resumen'!$A$1:$B$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1844,12 +1844,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CP-MATH-001</t>
+          <t>CP-ENG-005</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Core Math</t>
+          <t>Engines</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1864,22 +1864,22 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Escalas y coordenadas SVG</t>
+          <t>Estructuras lineales generan pasos correctos</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Datos numericos</t>
+          <t>Stack, Queue y Linked List disponibles</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>dataset de barras</t>
+          <t>[1,2,3]</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Calcula posiciones y transiciones sin NaN</t>
+          <t>Genera pasos de insercion, recorrido/extraccion y estado final esperado</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1894,19 +1894,19 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>packages/core/src/math/__tests__/math.test.ts</t>
+          <t>packages/core/src/engines/__tests__/linear-structures.test.ts</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CP-VAL-001</t>
+          <t>CP-MATH-001</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Validadores</t>
+          <t>Core Math</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1916,27 +1916,27 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>HU-03</t>
+          <t>HU-04</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Dataset valido</t>
+          <t>Escalas y coordenadas SVG</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Valores enteros</t>
+          <t>Datos numericos</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>[1,2,3]</t>
+          <t>dataset de barras</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Valida sin errores</t>
+          <t>Calcula posiciones y transiciones sin NaN</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1951,14 +1951,14 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>packages/core/src/validators/__tests__/dataset.test.ts</t>
+          <t>packages/core/src/math/__tests__/math.test.ts</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CP-VAL-002</t>
+          <t>CP-VAL-001</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1978,22 +1978,22 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Dataset invalido</t>
+          <t>Dataset valido</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Valores nulos/no numericos</t>
+          <t>Valores enteros</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>[1,null,'x']</t>
+          <t>[1,2,3]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Retorna errores claros</t>
+          <t>Valida sin errores</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2015,12 +2015,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CP-EJR-001</t>
+          <t>CP-VAL-002</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Ejercicios</t>
+          <t>Validadores</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2030,27 +2030,27 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>RF-EJR</t>
+          <t>HU-03</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Listar ejercicios por algoritmo</t>
+          <t>Dataset invalido</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Algoritmo con ejercicios</t>
+          <t>Valores nulos/no numericos</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>algoritmoId</t>
+          <t>[1,null,'x']</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Retorna ejercicios sin respuesta sensible innecesaria</t>
+          <t>Retorna errores claros</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2065,14 +2065,14 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>src/exercises/exercises.service.spec.ts</t>
+          <t>packages/core/src/validators/__tests__/dataset.test.ts</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CP-EJR-002</t>
+          <t>CP-EJR-001</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2092,22 +2092,22 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Responder correctamente</t>
+          <t>Listar ejercicios por algoritmo</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Ejercicio existente</t>
+          <t>Algoritmo con ejercicios</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>respuesta correcta</t>
+          <t>algoritmoId</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>correcto=true, puntosGanados, feedback y feedbackPositivo</t>
+          <t>Retorna ejercicios sin respuesta sensible innecesaria</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Critica</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2129,7 +2129,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CP-EJR-003</t>
+          <t>CP-EJR-002</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Responder incorrectamente</t>
+          <t>Responder correctamente</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2159,12 +2159,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>respuesta incorrecta</t>
+          <t>respuesta correcta</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>correcto=false, puntosGanados=0, feedback y feedbackNegativo</t>
+          <t>correcto=true, puntosGanados, feedback y feedbackPositivo</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Critica</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CP-EJR-004</t>
+          <t>CP-EJR-003</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2206,22 +2206,22 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Actualizar racha</t>
+          <t>Responder incorrectamente</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>ultimaActividad ayer/hoy/&gt;2 dias</t>
+          <t>Ejercicio existente</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>fechas limite</t>
+          <t>respuesta incorrecta</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Incrementa, mantiene o reinicia racha segun regla</t>
+          <t>correcto=false, puntosGanados=0, feedback y feedbackNegativo</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Critica</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -2243,7 +2243,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CP-EJR-005</t>
+          <t>CP-EJR-004</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>Unitaria</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2263,22 +2263,22 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Flujo ejercicio HTTP</t>
+          <t>Actualizar racha</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Token valido</t>
+          <t>ultimaActividad ayer/hoy/&gt;2 dias</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>GET y POST responder</t>
+          <t>fechas limite</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Respuesta contiene correcto, feedback, puntos y progreso</t>
+          <t>Incrementa, mantiene o reinicia racha segun regla</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2293,49 +2293,49 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>test/exercises.e2e-spec.ts</t>
+          <t>src/exercises/exercises.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CP-PRG-001</t>
+          <t>CP-EJR-005</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Progreso</t>
+          <t>Ejercicios</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Unitaria</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>RF-PRG</t>
+          <t>RF-EJR</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Consultar progreso</t>
+          <t>Flujo ejercicio HTTP</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Progreso existente</t>
+          <t>Token valido</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>usuarioId</t>
+          <t>GET y POST responder</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Retorna puntos, nivel, racha, ranking e insignias</t>
+          <t>Respuesta contiene correcto, feedback, puntos y progreso</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2345,19 +2345,19 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Critica</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>src/progress/progress.service.spec.ts</t>
+          <t>test/exercises.e2e-spec.ts</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>CP-PRG-002</t>
+          <t>CP-PRG-001</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2377,22 +2377,22 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Ranking paginado</t>
+          <t>Consultar progreso</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Usuarios con progreso</t>
+          <t>Progreso existente</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>limit/offset</t>
+          <t>usuarioId</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Retorna ranking ordenado y total</t>
+          <t>Retorna puntos, nivel, racha, ranking e insignias</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2414,7 +2414,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>CP-PRG-003</t>
+          <t>CP-PRG-002</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>Unitaria</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2434,22 +2434,22 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>GET progreso y ranking</t>
+          <t>Ranking paginado</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Token valido</t>
+          <t>Usuarios con progreso</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>/api/progreso/me y /ranking</t>
+          <t>limit/offset</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Respuestas 200 y filtros defensivos</t>
+          <t>Retorna ranking ordenado y total</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2464,49 +2464,49 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>test/progress.e2e-spec.ts</t>
+          <t>src/progress/progress.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CP-INS-001</t>
+          <t>CP-PRG-003</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Insignias</t>
+          <t>Progreso</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Unitaria</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>RF-INS</t>
+          <t>RF-PRG</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Listar insignias</t>
+          <t>GET progreso y ranking</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Seed de insignias</t>
+          <t>Token valido</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>sin parametros</t>
+          <t>/api/progreso/me y /ranking</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Retorna insignias disponibles</t>
+          <t>Respuestas 200 y filtros defensivos</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2516,19 +2516,19 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>src/badges/badges.service.spec.ts</t>
+          <t>test/progress.e2e-spec.ts</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>CP-INS-002</t>
+          <t>CP-INS-001</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2548,22 +2548,22 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Otorgar insignia por criterio</t>
+          <t>Listar insignias</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Progreso cumple criterio</t>
+          <t>Seed de insignias</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>usuarioId</t>
+          <t>sin parametros</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Crea ProgresoInsignia sin duplicar</t>
+          <t>Retorna insignias disponibles</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -2585,12 +2585,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>CP-SYNC-001</t>
+          <t>CP-INS-002</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Sync</t>
+          <t>Insignias</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2600,27 +2600,27 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>RF-SYNC</t>
+          <t>RF-INS</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Sincronizar sesiones offline</t>
+          <t>Otorgar insignia por criterio</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Payload offline valido</t>
+          <t>Progreso cumple criterio</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>sesiones[]</t>
+          <t>usuarioId</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Registra sesiones y puntosActualizados</t>
+          <t>Crea ProgresoInsignia sin duplicar</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2635,19 +2635,19 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>src/sync/sync.service.spec.ts</t>
+          <t>src/badges/badges.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>CP-OFF-001</t>
+          <t>CP-SYNC-001</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Sync</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2657,27 +2657,27 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>RF-OFF</t>
+          <t>RF-SYNC</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Listar modulos offline</t>
+          <t>Sincronizar sesiones offline</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Algoritmos activos</t>
+          <t>Payload offline valido</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>usuarioId</t>
+          <t>sesiones[]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Retorna algoritmoId,nombre,tamanoKB,version,descargado</t>
+          <t>Registra sesiones y puntosActualizados</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2687,19 +2687,19 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>src/offline/offline.service.spec.ts</t>
+          <t>src/sync/sync.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>CP-OFF-002</t>
+          <t>CP-OFF-001</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Unitaria/E2E</t>
+          <t>Unitaria</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2719,22 +2719,22 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Descargar modulo</t>
+          <t>Listar modulos offline</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Algoritmo existente</t>
+          <t>Algoritmos activos</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>algoritmoId</t>
+          <t>usuarioId</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Retorna algoritmoId, version, meta, pseudocode y ejercicios</t>
+          <t>Retorna algoritmoId,nombre,tamanoKB,version,descargado</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2744,54 +2744,54 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>src/offline/offline.service.spec.ts; test/learning-support.e2e-spec.ts</t>
+          <t>src/offline/offline.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>CP-DIAG-001</t>
+          <t>CP-OFF-002</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Diagnostico</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Unitaria</t>
+          <t>Unitaria/E2E</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>RF-DIAG</t>
+          <t>RF-OFF</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Listar preguntas</t>
+          <t>Descargar modulo</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Preguntas seed</t>
+          <t>Algoritmo existente</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>sin parametros</t>
+          <t>algoritmoId</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Retorna preguntas y opciones</t>
+          <t>Retorna algoritmoId, version, meta, pseudocode y ejercicios</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2801,19 +2801,19 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>src/diagnostics/diagnostics.service.spec.ts</t>
+          <t>src/offline/offline.service.spec.ts; test/learning-support.e2e-spec.ts</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>CP-DIAG-002</t>
+          <t>CP-DIAG-001</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2833,22 +2833,22 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Evaluar diagnostico</t>
+          <t>Listar preguntas</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Respuestas enviadas</t>
+          <t>Preguntas seed</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>indices seleccionados</t>
+          <t>sin parametros</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Calcula puntaje, guarda resultado y genera ruta</t>
+          <t>Retorna preguntas y opciones</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -2870,12 +2870,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>CP-RUTA-001</t>
+          <t>CP-DIAG-002</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Ruta Aprendizaje</t>
+          <t>Diagnostico</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2885,27 +2885,27 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>RF-RUTA</t>
+          <t>RF-DIAG</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Consultar ruta personalizada</t>
+          <t>Evaluar diagnostico</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Usuario con diagnostico/ruta</t>
+          <t>Respuestas enviadas</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>usuarioId</t>
+          <t>indices seleccionados</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Retorna algoritmos sugeridos en orden</t>
+          <t>Calcula puntaje, guarda resultado y genera ruta</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -2915,54 +2915,54 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>src/learning-path/learning-path.service.spec.ts</t>
+          <t>src/diagnostics/diagnostics.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CP-LRN-001</t>
+          <t>CP-RUTA-001</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Soporte Aprendizaje</t>
+          <t>Ruta Aprendizaje</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>Unitaria</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>RF-DIAG/RF-RUTA</t>
+          <t>RF-RUTA</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Evaluar diagnostico y consultar ruta HTTP</t>
+          <t>Consultar ruta personalizada</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Token valido y preguntas diagnosticas</t>
+          <t>Usuario con diagnostico/ruta</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>GET preguntas, POST evaluar, GET ruta</t>
+          <t>usuarioId</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Respuestas 200/201 y ruta con algoritmos sugeridos</t>
+          <t>Retorna algoritmos sugeridos en orden</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2972,24 +2972,24 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>test/learning-support.e2e-spec.ts</t>
+          <t>src/learning-path/learning-path.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>CP-LRN-002</t>
+          <t>CP-LRN-001</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Insignias</t>
+          <t>Soporte Aprendizaje</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2999,27 +2999,27 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>RF-INS</t>
+          <t>RF-DIAG/RF-RUTA</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Consultar insignias HTTP</t>
+          <t>Evaluar diagnostico y consultar ruta HTTP</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Token valido</t>
+          <t>Token valido y preguntas diagnosticas</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>GET /api/insignias y /api/insignias/me</t>
+          <t>GET preguntas, POST evaluar, GET ruta</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Lista insignias disponibles y estado del usuario</t>
+          <t>Respuestas 200/201 y ruta con algoritmos sugeridos</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -3041,12 +3041,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>CP-LRN-003</t>
+          <t>CP-LRN-002</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Insignias</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3056,27 +3056,27 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>RF-OFF</t>
+          <t>RF-INS</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Listar y descargar modulo offline HTTP</t>
+          <t>Consultar insignias HTTP</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Token valido y algoritmos activos</t>
+          <t>Token valido</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>GET /api/modules/offline y /download</t>
+          <t>GET /api/insignias y /api/insignias/me</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Retorna meta, pseudocode y ejercicios del modulo</t>
+          <t>Lista insignias disponibles y estado del usuario</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3098,12 +3098,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>CP-LRN-004</t>
+          <t>CP-LRN-003</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Seguridad API</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3113,27 +3113,27 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>RF-AUTH</t>
+          <t>RF-OFF</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Proteger endpoints de aprendizaje</t>
+          <t>Listar y descargar modulo offline HTTP</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Sin token JWT</t>
+          <t>Token valido y algoritmos activos</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>GET endpoints protegidos</t>
+          <t>GET /api/modules/offline y /download</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Retorna 401 Unauthorized</t>
+          <t>Retorna meta, pseudocode y ejercicios del modulo</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Critica</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -3155,62 +3155,347 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>CP-LRN-004</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Seguridad API</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>RF-AUTH</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Proteger endpoints de aprendizaje</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Sin token JWT</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>GET endpoints protegidos</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Retorna 401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Critica</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>test/learning-support.e2e-spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
           <t>CP-FE-SVC-001</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>Contratos FE</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Unitaria</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>RF-CONTRATOS</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>Consumir contratos API desde frontend</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>apiClient mockeado</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>ranking, sync, offline, ejercicios</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Valida endpoints y forma ranking/total, completada, algoritmoId/version y feedback</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>PASO</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>src/services/__tests__/contract-shapes.test.ts</t>
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-SVC-002</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Servicios FE</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>RF-CONTRATOS</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Servicios frontend usan endpoints y payloads correctos</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>apiClient mockeado</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>auth, biblioteca, simulaciones, ejercicios, progreso, diagnostico, offline</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Valida rutas publicas/protegidas y payloads enviados al backend</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>src/services/__tests__/api-services.test.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-UTL-001</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Utilidades FE</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>RF-UX</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Validadores de formularios y dataset</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Funciones puras disponibles</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>nombre, correo, password, rol, dataset y velocidad</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Acepta entradas validas y rechaza clases invalidas con mensajes claros</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>src/utils/__tests__/validators.test.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-UTL-002</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Utilidades FE</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>RF-UX</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Formateadores de interfaz</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Funciones puras disponibles</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>puntos, porcentajes, tamanos, velocidades, duraciones y descripciones</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Formatea valores para UI en locale es-MX y trunca descripciones</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>src/utils/__tests__/formatters.test.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-XP-001</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Gamificacion FE</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>RF-PRG</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Calculo local de XP, nivel y tier</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Funciones puras disponibles</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>puntos acumulados y niveles limite</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Respeta formula cuadratica, nivel maximo, progreso y tier esperado</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>src/utils/__tests__/xp.utils.test.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K48"/>
+  <autoFilter ref="A1:K53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3702,7 +3987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3922,7 +4207,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>CP-ENG-001, CP-ENG-002, CP-ENG-003, CP-ENG-004</t>
+          <t>CP-ENG-001, CP-ENG-002, CP-ENG-003, CP-ENG-004, CP-ENG-005</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -4022,17 +4307,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>RF-DIAG</t>
+          <t>RF-CONTRATOS</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Diagnostico</t>
+          <t>Servicios FE</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>CP-DIAG-001, CP-DIAG-002</t>
+          <t>CP-FE-SVC-002</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -4044,17 +4329,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>RF-DIAG/RF-RUTA</t>
+          <t>RF-DIAG</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Soporte Aprendizaje</t>
+          <t>Diagnostico</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>CP-LRN-001</t>
+          <t>CP-DIAG-001, CP-DIAG-002</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -4066,17 +4351,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>RF-EJR</t>
+          <t>RF-DIAG/RF-RUTA</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Ejercicios</t>
+          <t>Soporte Aprendizaje</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>CP-EJR-001, CP-EJR-002, CP-EJR-003, CP-EJR-004, CP-EJR-005</t>
+          <t>CP-LRN-001</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -4088,17 +4373,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>RF-INS</t>
+          <t>RF-EJR</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Insignias</t>
+          <t>Ejercicios</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>CP-INS-001, CP-INS-002, CP-LRN-002</t>
+          <t>CP-EJR-001, CP-EJR-002, CP-EJR-003, CP-EJR-004, CP-EJR-005</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -4110,17 +4395,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>RF-OFF</t>
+          <t>RF-INS</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Insignias</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>CP-OFF-001, CP-OFF-002, CP-LRN-003</t>
+          <t>CP-INS-001, CP-INS-002, CP-LRN-002</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -4132,17 +4417,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>RF-PRG</t>
+          <t>RF-OFF</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Progreso</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>CP-PRG-001, CP-PRG-002, CP-PRG-003</t>
+          <t>CP-OFF-001, CP-OFF-002, CP-LRN-003</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -4154,17 +4439,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>RF-RUTA</t>
+          <t>RF-PRG</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Ruta Aprendizaje</t>
+          <t>Gamificacion FE</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>CP-RUTA-001</t>
+          <t>CP-FE-XP-001</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4176,17 +4461,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>RF-SYNC</t>
+          <t>RF-PRG</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Sync</t>
+          <t>Progreso</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>CP-SYNC-001</t>
+          <t>CP-PRG-001, CP-PRG-002, CP-PRG-003</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -4198,27 +4483,93 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>RF-RUTA</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Ruta Aprendizaje</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>CP-RUTA-001</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Automatizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>RF-SYNC</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Sync</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>CP-SYNC-001</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Automatizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>RF-USR</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Usuarios</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>CP-USR-001, CP-USR-002</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Automatizado</t>
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>RF-UX</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Utilidades FE</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-UTL-001, CP-FE-UTL-002</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Automatizado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D23"/>
+  <autoFilter ref="A1:D26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4229,7 +4580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4824,7 +5175,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>packages/core/src/math/__tests__/math.test.ts</t>
+          <t>packages/core/src/engines/__tests__/linear-structures.test.ts</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -4837,7 +5188,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Escalas, coordenadas, transiciones</t>
+          <t>Stack, Queue y Linked List</t>
         </is>
       </c>
     </row>
@@ -4849,7 +5200,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>packages/core/src/validators/__tests__/dataset.test.ts</t>
+          <t>packages/core/src/math/__tests__/math.test.ts</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -4858,11 +5209,11 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Validacion de datasets</t>
+          <t>Escalas, coordenadas, transiciones</t>
         </is>
       </c>
     </row>
@@ -4874,25 +5225,150 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
+          <t>packages/core/src/validators/__tests__/dataset.test.ts</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Validacion de datasets</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
           <t>src/services/__tests__/contract-shapes.test.ts</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Unitaria</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="n">
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Contratos frontend para ranking, ejercicios, offline y sync</t>
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>src/services/__tests__/api-services.test.ts</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Endpoints y payloads de servicios frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>src/utils/__tests__/validators.test.ts</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Validadores de auth, dataset y velocidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>src/utils/__tests__/formatters.test.ts</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Formato de numeros, fechas relativas, velocidad y texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>src/utils/__tests__/xp.utils.test.ts</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Unitaria</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Formula XP, nivel, progreso y tiers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E26"/>
+  <autoFilter ref="A1:E31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4929,7 +5405,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
@@ -4939,7 +5415,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>162</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4">
@@ -4974,7 +5450,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>7 suites / 35 tests pasados</t>
+          <t>12 suites / 66 tests pasados</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update testing evidence for Playwright coverage
</commit_message>
<xml_diff>
--- a/pruebas/3.2-Casos-de-Prueba-BrainSort.xlsx
+++ b/pruebas/3.2-Casos-de-Prueba-BrainSort.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Prueba'!$A$1:$K$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Prueba'!$A$1:$K$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Equivalencia y Limites'!$A$1:$L$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trazabilidad'!$A$1:$D$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automatizacion'!$A$1:$E$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Resumen'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trazabilidad'!$A$1:$D$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automatizacion'!$A$1:$E$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Resumen'!$A$1:$B$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3494,8 +3494,179 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-E2E-001</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Login UI</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>E2E Web</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>RF-AUTH</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Login desde pantalla web</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Expo Web levantado y API mockeada</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>correo y contrasena validos</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Autentica y muestra navegacion principal</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Critica</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>e2e/app-flows.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-E2E-002</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Ruta UI</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>E2E Web</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>RF-RUTA</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Ruta de aprendizaje visible</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Sesion dev activa y API mockeada</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>click en tab Ruta</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Muestra secuencia recomendada con algoritmos</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>e2e/app-flows.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-E2E-003</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Perfil UI</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>E2E Web</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>RF-USR</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Perfil muestra y actualiza nombre</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Sesion dev activa y API mockeada</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>editar nombre y guardar</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Muestra datos de usuario y persiste nombre local editado</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>e2e/app-flows.spec.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K53"/>
+  <autoFilter ref="A1:K56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3987,7 +4158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4268,12 +4439,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Seguridad API</t>
+          <t>Login UI</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>CP-LRN-004</t>
+          <t>CP-FE-E2E-001</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -4285,17 +4456,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>RF-CONTRATOS</t>
+          <t>RF-AUTH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Contratos FE</t>
+          <t>Seguridad API</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>CP-FE-SVC-001</t>
+          <t>CP-LRN-004</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -4312,12 +4483,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Servicios FE</t>
+          <t>Contratos FE</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>CP-FE-SVC-002</t>
+          <t>CP-FE-SVC-001</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -4329,17 +4500,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>RF-DIAG</t>
+          <t>RF-CONTRATOS</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Diagnostico</t>
+          <t>Servicios FE</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>CP-DIAG-001, CP-DIAG-002</t>
+          <t>CP-FE-SVC-002</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -4351,17 +4522,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>RF-DIAG/RF-RUTA</t>
+          <t>RF-DIAG</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Soporte Aprendizaje</t>
+          <t>Diagnostico</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>CP-LRN-001</t>
+          <t>CP-DIAG-001, CP-DIAG-002</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -4373,17 +4544,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>RF-EJR</t>
+          <t>RF-DIAG/RF-RUTA</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Ejercicios</t>
+          <t>Soporte Aprendizaje</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>CP-EJR-001, CP-EJR-002, CP-EJR-003, CP-EJR-004, CP-EJR-005</t>
+          <t>CP-LRN-001</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -4395,17 +4566,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>RF-INS</t>
+          <t>RF-EJR</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Insignias</t>
+          <t>Ejercicios</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>CP-INS-001, CP-INS-002, CP-LRN-002</t>
+          <t>CP-EJR-001, CP-EJR-002, CP-EJR-003, CP-EJR-004, CP-EJR-005</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -4417,17 +4588,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>RF-OFF</t>
+          <t>RF-INS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Insignias</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>CP-OFF-001, CP-OFF-002, CP-LRN-003</t>
+          <t>CP-INS-001, CP-INS-002, CP-LRN-002</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -4439,17 +4610,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>RF-PRG</t>
+          <t>RF-OFF</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Gamificacion FE</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>CP-FE-XP-001</t>
+          <t>CP-OFF-001, CP-OFF-002, CP-LRN-003</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4466,12 +4637,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Progreso</t>
+          <t>Gamificacion FE</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>CP-PRG-001, CP-PRG-002, CP-PRG-003</t>
+          <t>CP-FE-XP-001</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -4483,17 +4654,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>RF-RUTA</t>
+          <t>RF-PRG</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Ruta Aprendizaje</t>
+          <t>Progreso</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>CP-RUTA-001</t>
+          <t>CP-PRG-001, CP-PRG-002, CP-PRG-003</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -4505,17 +4676,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>RF-SYNC</t>
+          <t>RF-RUTA</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Sync</t>
+          <t>Ruta Aprendizaje</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>CP-SYNC-001</t>
+          <t>CP-RUTA-001</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4527,17 +4698,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>RF-USR</t>
+          <t>RF-RUTA</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Usuarios</t>
+          <t>Ruta UI</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>CP-USR-001, CP-USR-002</t>
+          <t>CP-FE-E2E-002</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -4549,27 +4720,93 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>RF-SYNC</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Sync</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>CP-SYNC-001</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Automatizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>RF-USR</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Perfil UI</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>CP-FE-E2E-003</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Automatizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>RF-USR</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Usuarios</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CP-USR-001, CP-USR-002</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Automatizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>RF-UX</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Utilidades FE</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>CP-FE-UTL-001, CP-FE-UTL-002</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Automatizado</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D26"/>
+  <autoFilter ref="A1:D29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4580,7 +4817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5367,8 +5604,33 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>e2e/app-flows.spec.ts</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>E2E Web</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Login, ruta de aprendizaje y perfil en Expo Web con Playwright</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E31"/>
+  <autoFilter ref="A1:E32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5379,7 +5641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5405,7 +5667,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3">
@@ -5415,7 +5677,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4">
@@ -5457,41 +5719,53 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Rama evidencia</t>
+          <t>Frontend E2E Web</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>API feature/unit-tests-qa; APP feature/contract-consistency-fixes</t>
+          <t>1 suite Playwright / 3 tests pasados</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Commit API</t>
+          <t>Rama evidencia</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>86b4413 base + cambios locales de contratos</t>
+          <t>API feature/unit-tests-qa; APP feature/contract-consistency-fixes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Commit API</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>86b4413 base + cambios locales de contratos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Commit APP</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>b66290b base dev + cambios locales de contratos</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>